<commit_message>
Strip all Excel templates to headers only (remove 3,659 data rows)
Removed all internal data from 8 Excel files across 22 sheets.
Files now serve as clean structural templates showing column layout only.
</commit_message>
<xml_diff>
--- a/05-Maintenance-Scheduling/Schedule-Templates/90 Day Outlook_IEM.xlsx
+++ b/05-Maintenance-Scheduling/Schedule-Templates/90 Day Outlook_IEM.xlsx
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="MM/DD/YYYY"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="MM/DD/YYYY"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -73,7 +72,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -441,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -538,351 +537,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>PDX97</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>[GLOBAL] AMCOP 36M PM V1.0</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>46235</v>
-      </c>
-      <c r="F2" s="3" t="n">
-        <v>46180</v>
-      </c>
-      <c r="G2" s="3" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="n"/>
-      <c r="M2" s="2" t="n"/>
-      <c r="N2" s="2" t="n"/>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>MCM Needed (&lt;60d)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>PDX58</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>[GLOBAL] AMCOP 36M PM V1.0</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>46274</v>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>46219</v>
-      </c>
-      <c r="G3" s="3" t="n">
-        <v>46329</v>
-      </c>
-      <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="n"/>
-      <c r="J3" s="2" t="n"/>
-      <c r="K3" s="2" t="n"/>
-      <c r="L3" s="2" t="n"/>
-      <c r="M3" s="2" t="n"/>
-      <c r="N3" s="2" t="n"/>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>MCM Needed (&lt;90d)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>PDX55</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>[GLOBAL] BACKSTOPPING CONTROL PANEL 36M PM V1.0</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>46296</v>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>46241</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>46351</v>
-      </c>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="n"/>
-      <c r="J4" s="2" t="n"/>
-      <c r="K4" s="2" t="n"/>
-      <c r="L4" s="2" t="n"/>
-      <c r="M4" s="2" t="n"/>
-      <c r="N4" s="2" t="n"/>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>MCM Needed (&lt;90d)</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010091BDD0564093794395D1C5349333D5B2" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1452c3346e618de032dde90eee50b30b">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bf647356-47fe-4b60-9e60-e582934d7a8a" xmlns:ns3="6741c247-c55f-4916-bd12-c6d420d6ec93" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1641523bb374e78ed969369e342c04e6" ns2:_="" ns3:_="">
-    <xsd:import namespace="bf647356-47fe-4b60-9e60-e582934d7a8a"/>
-    <xsd:import namespace="6741c247-c55f-4916-bd12-c6d420d6ec93"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="bf647356-47fe-4b60-9e60-e582934d7a8a" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="37839dc8-c537-42b6-a5a9-a537040d25bb" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="6741c247-c55f-4916-bd12-c6d420d6ec93" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{733ce214-3297-436b-9b8a-fd4769f86a2c}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="6741c247-c55f-4916-bd12-c6d420d6ec93">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6741c247-c55f-4916-bd12-c6d420d6ec93" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bf647356-47fe-4b60-9e60-e582934d7a8a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{49D29FAC-84D5-46E3-8384-B8CC1545B621}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6EBA1814-4FB4-4684-A6FB-816B5D8BA75C}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6E2203F-B842-4CDF-94BA-817DBBD96501}"/>
 </file>
</xml_diff>